<commit_message>
Add a specific examples in the report, clear typos
</commit_message>
<xml_diff>
--- a/compiler_practice_counts.xlsx
+++ b/compiler_practice_counts.xlsx
@@ -666,18 +666,18 @@
         <v>-75.8620689655172</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K5" s="9" t="n">
         <v>7</v>
       </c>
       <c r="L5" s="9" t="n">
         <f aca="false">K5-J5</f>
-        <v>-21</v>
+        <v>-22</v>
       </c>
       <c r="M5" s="10" t="n">
         <f aca="false">L5/J5*100</f>
-        <v>-75</v>
+        <v>-75.8620689655172</v>
       </c>
       <c r="N5" s="11" t="s">
         <v>3</v>
@@ -819,15 +819,15 @@
         <v>65</v>
       </c>
       <c r="K8" s="9" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="L8" s="9" t="n">
         <f aca="false">K8-J8</f>
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="M8" s="10" t="n">
         <f aca="false">L8/J8*100</f>
-        <v>-3.07692307692308</v>
+        <v>1.53846153846154</v>
       </c>
       <c r="N8" s="11" t="s">
         <v>4</v>

</xml_diff>